<commit_message>
Update fulltext_source for 89 papers previously misrecorded as abstract-only
HTML extraction strategy recovered full text via DOI/Unpaywall HTML for papers
where PMC blocked XML download or PDF was unavailable. Classifications unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NF_Guidelines_Curated.xlsx
+++ b/NF_Guidelines_Curated.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Classified Papers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary Counts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="By Year" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classified Papers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary Counts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Year" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -806,7 +806,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.5858/arpa.2015-0314-RA</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00381-016-3093-3</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://nrs.harvard.edu/urn-3:HUL.InstRepos:32725810</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/5578356</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/5578359</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://nrs.harvard.edu/urn-3:HUL.InstRepos:32725809</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://dspace.library.uu.nl/handle/1874/363421</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://research.manchester.ac.uk/en/publications/3229ea40-51a2-4efb-bd8b-b65ca0442ef1</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1055/s-0037-1608814</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1055/s-0037-1608869</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.5152/iao.2018.5348</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00381-018-3833-7</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Suerink Wimmer 2018 CMMRD as diff of NF1.pdf</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11547-018-0955-7</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:e46.pdf</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
@@ -7241,7 +7241,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1055/s-0039-1691830</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10143-019-01135-y</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11060-019-03234-8</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11060-019-03247-3</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00256-019-03290-1</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://research.manchester.ac.uk/en/publications/216f3071-4682-4a6a-be22-d423c3fbcf75</t>
         </is>
       </c>
       <c r="F132" s="3" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00405-019-05741-w</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -9339,7 +9339,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1055/s-0040-1710524</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12020-020-02351-z</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Journal of Genetic Counseling - 2020 - Radtke - Genetic Counseling for Neurofibromatosis 1 Neurofibromatosis 2 and.pdf</t>
         </is>
       </c>
       <c r="F164" s="3" t="inlineStr">
@@ -10025,7 +10025,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00381-020-04706-3</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -10475,7 +10475,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12328-020-01227-z</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/7486535</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://hdl.handle.net/10072/416369</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/8246828</t>
         </is>
       </c>
       <c r="F195" s="2" t="inlineStr">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Aronson 2021 Diagnostic criteria for CMMRD international consensus group.pdf</t>
         </is>
       </c>
       <c r="F202" s="3" t="inlineStr">
@@ -11857,7 +11857,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00105-021-04779-4</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
@@ -11957,7 +11957,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11906-021-01136-7</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00117-021-00861-z</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -12747,7 +12747,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/8594008</t>
         </is>
       </c>
       <c r="F224" s="3" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/8594001</t>
         </is>
       </c>
       <c r="F225" s="3" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/8594004</t>
         </is>
       </c>
       <c r="F231" s="2" t="inlineStr">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://pure.eur.nl/en/publications/8118ce3b-c70d-4b0b-b224-20b4e97efc4f</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00117-021-00892-6</t>
         </is>
       </c>
       <c r="F234" s="2" t="inlineStr">
@@ -13501,7 +13501,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PMC XML</t>
         </is>
       </c>
       <c r="F235" s="2" t="inlineStr">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12070-020-02321-x</t>
         </is>
       </c>
       <c r="F239" s="2" t="inlineStr">
@@ -14251,7 +14251,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://hdl.handle.net/10138/351298</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://hdl.handle.net/10072/426076</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
@@ -14983,7 +14983,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://www.ncbi.nlm.nih.gov/pmc/articles/9018953</t>
         </is>
       </c>
       <c r="F264" s="2" t="inlineStr">
@@ -16251,7 +16251,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11060-022-04104-6</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
@@ -16601,7 +16601,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00117-022-01059-7</t>
         </is>
       </c>
       <c r="F293" s="3" t="inlineStr">
@@ -16983,7 +16983,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11845-022-03184-7</t>
         </is>
       </c>
       <c r="F300" s="2" t="inlineStr">
@@ -17773,7 +17773,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12070-021-02900-6</t>
         </is>
       </c>
       <c r="F315" s="2" t="inlineStr">
@@ -17873,7 +17873,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Halliday et al 2023 Updated protocol for genetic testing screening and clinical management of indiv at risk of NF2.SWN.pdf</t>
         </is>
       </c>
       <c r="F317" s="3" t="inlineStr">
@@ -18013,7 +18013,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00586-023-07600-z</t>
         </is>
       </c>
       <c r="F319" s="2" t="inlineStr">
@@ -18113,7 +18113,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://hal.inrae.fr/hal-04246685/document</t>
         </is>
       </c>
       <c r="F321" s="2" t="inlineStr">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1245/s10434-023-13519-y</t>
         </is>
       </c>
       <c r="F326" s="2" t="inlineStr">
@@ -18413,7 +18413,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Koza 2023 Consensus recommendations on counselling in Phelan-McDermid ring 22.pdf</t>
         </is>
       </c>
       <c r="F327" s="3" t="inlineStr">
@@ -18831,7 +18831,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12070-022-03229-4</t>
         </is>
       </c>
       <c r="F334" s="2" t="inlineStr">
@@ -18931,7 +18931,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10689-023-00340-5</t>
         </is>
       </c>
       <c r="F336" s="2" t="inlineStr">
@@ -19427,7 +19427,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://ojs.ptbioch.edu.pl/index.php/abp/article/download/6955/5839</t>
         </is>
       </c>
       <c r="F346" s="2" t="inlineStr">
@@ -19527,7 +19527,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PMC XML</t>
         </is>
       </c>
       <c r="F348" s="3" t="inlineStr">
@@ -20101,7 +20101,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11912-023-01451-z</t>
         </is>
       </c>
       <c r="F357" s="2" t="inlineStr">
@@ -20201,7 +20201,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PMC XML</t>
         </is>
       </c>
       <c r="F359" s="2" t="inlineStr">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00256-023-04511-4</t>
         </is>
       </c>
       <c r="F361" s="2" t="inlineStr">
@@ -20451,7 +20451,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00586-023-08039-y</t>
         </is>
       </c>
       <c r="F364" s="2" t="inlineStr">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1055/s-0043-1777702</t>
         </is>
       </c>
       <c r="F365" s="2" t="inlineStr">
@@ -20751,7 +20751,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:https://discovery.ucl.ac.uk/10185874/2/Jacques_Consensus%20framework%20for%20conducting%20phase%20I_II%20clinical%20trials%20for%20children%2C%20adolescents%2C%20and%20young%20adults%20with%20pediatric%20low-grade%20glioma_AAM.pdf</t>
         </is>
       </c>
       <c r="F370" s="3" t="inlineStr">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11136-023-03596-7</t>
         </is>
       </c>
       <c r="F373" s="2" t="inlineStr">
@@ -21011,7 +21011,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10143-024-02305-3</t>
         </is>
       </c>
       <c r="F374" s="2" t="inlineStr">
@@ -21347,7 +21347,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11060-024-04617-2</t>
         </is>
       </c>
       <c r="F380" s="2" t="inlineStr">
@@ -21547,7 +21547,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00586-024-08194-w</t>
         </is>
       </c>
       <c r="F384" s="2" t="inlineStr">
@@ -21979,7 +21979,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:http://urn.kb.se/resolve?urn=urn:nbn:se:uu:diva-577770</t>
         </is>
       </c>
       <c r="F392" s="2" t="inlineStr">
@@ -22479,7 +22479,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00330-024-10885-3</t>
         </is>
       </c>
       <c r="F402" s="2" t="inlineStr">
@@ -23395,7 +23395,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10143-024-02889-w</t>
         </is>
       </c>
       <c r="F416" s="2" t="inlineStr">
@@ -24035,7 +24035,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s12070-024-04910-6</t>
         </is>
       </c>
       <c r="F428" s="2" t="inlineStr">
@@ -24385,7 +24385,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00431-024-05825-8</t>
         </is>
       </c>
       <c r="F435" s="2" t="inlineStr">
@@ -24585,7 +24585,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>PDF:Dtsch_Arztebl_Int-122_071.pdf</t>
         </is>
       </c>
       <c r="F439" s="3" t="inlineStr">
@@ -25359,7 +25359,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00403-025-04056-7</t>
         </is>
       </c>
       <c r="F452" s="2" t="inlineStr">
@@ -25709,7 +25709,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://research.manchester.ac.uk/en/publications/0ee1dd1c-7856-4ae3-95ef-b487ee6a4ab4</t>
         </is>
       </c>
       <c r="F459" s="2" t="inlineStr">
@@ -25809,7 +25809,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10143-025-03519-9</t>
         </is>
       </c>
       <c r="F461" s="2" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11033-025-10431-4</t>
         </is>
       </c>
       <c r="F463" s="2" t="inlineStr">
@@ -26409,7 +26409,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s10147-025-02793-3</t>
         </is>
       </c>
       <c r="F473" s="2" t="inlineStr">
@@ -26559,7 +26559,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1038/s41434-025-00542-9</t>
         </is>
       </c>
       <c r="F476" s="2" t="inlineStr">
@@ -27289,7 +27289,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1038/s41416-025-03151-w</t>
         </is>
       </c>
       <c r="F489" s="2" t="inlineStr">
@@ -27725,7 +27725,7 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00405-025-09734-w</t>
         </is>
       </c>
       <c r="F497" s="2" t="inlineStr">
@@ -27875,7 +27875,7 @@
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11523-025-01176-y</t>
         </is>
       </c>
       <c r="F500" s="2" t="inlineStr">
@@ -27925,7 +27925,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1038/s41388-025-03617-4</t>
         </is>
       </c>
       <c r="F501" s="2" t="inlineStr">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s00431-025-06611-w</t>
         </is>
       </c>
       <c r="F502" s="2" t="inlineStr">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:doi:10.1007/s11060-025-05335-z</t>
         </is>
       </c>
       <c r="F521" s="2" t="inlineStr">
@@ -29215,7 +29215,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://doi.org/10.1038/s41431-026-02014-z</t>
         </is>
       </c>
       <c r="F526" s="2" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://cris.maastrichtuniversity.nl/en/publications/aeffa29c-94dc-4793-a566-de2d984aee9e</t>
         </is>
       </c>
       <c r="F529" s="2" t="inlineStr">
@@ -29697,7 +29697,7 @@
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://pure.eur.nl/en/publications/9055de50-f17f-4d60-8149-6cd815b0c964</t>
         </is>
       </c>
       <c r="F535" s="2" t="inlineStr">
@@ -29897,7 +29897,7 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>abstract_only</t>
+          <t>HTML:https://doi.org/10.1186/s13256-026-06002-1</t>
         </is>
       </c>
       <c r="F539" s="2" t="inlineStr">

</xml_diff>